<commit_message>
static dataframes for benchmark + visualisation answers
</commit_message>
<xml_diff>
--- a/visualization_benchmark_results.xlsx
+++ b/visualization_benchmark_results.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P6"/>
+  <dimension ref="A1:J21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,7 +446,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Expected Chart Type</t>
+          <t>Expected Chart</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -456,57 +456,27 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Datasets Used</t>
+          <t>Datasets</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Execution Success</t>
+          <t>Success</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>LLM Attempts</t>
+          <t>Attempts</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Readability Score</t>
+          <t>Code File</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Coherence Score</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Average Quality Score</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>Error Message</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Code File</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>Output Paths</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>Warnings Count</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>Final Answer</t>
+          <t>Error</t>
         </is>
       </c>
     </row>
@@ -547,36 +517,14 @@
       <c r="H2" t="n">
         <v>1</v>
       </c>
-      <c r="I2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>benchmarks\viz_results\generated_code\viz_001.py</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>reports\simple-timeseries.png</t>
-        </is>
-      </c>
-      <c r="O2" t="n">
-        <v>1</v>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>Generated 1 line chart from simple_ts dataset.</t>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -593,7 +541,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Plot the values as a bar chart.</t>
+          <t>Plot the number of occurrences of each category as a bar chart.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -617,36 +565,14 @@
       <c r="H3" t="n">
         <v>1</v>
       </c>
-      <c r="I3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>benchmarks\viz_results\generated_code\viz_002.py</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>reports\category-counts.png</t>
-        </is>
-      </c>
-      <c r="O3" t="n">
-        <v>1</v>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>Generated 1 bar chart from categorical</t>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -687,36 +613,14 @@
       <c r="H4" t="n">
         <v>1</v>
       </c>
-      <c r="I4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>benchmarks\viz_results\generated_code\viz_003.py</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>reports\measurements-scatter.png</t>
-        </is>
-      </c>
-      <c r="O4" t="n">
-        <v>1</v>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>Generated 1 scatter plot from measurements.</t>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -733,7 +637,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Plot multiple metrics on the same chart with legend and labels.</t>
+          <t>Plot the three metrics on the same chart with legend and labels.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -757,36 +661,14 @@
       <c r="H5" t="n">
         <v>1</v>
       </c>
-      <c r="I5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>benchmarks\viz_results\generated_code\viz_004.py</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>reports\multiple-metrics.png</t>
-        </is>
-      </c>
-      <c r="O5" t="n">
-        <v>1</v>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>Generated 1 figure with 2 subplots from wide_metrics.</t>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
     </row>
@@ -825,38 +707,737 @@
         <v>1</v>
       </c>
       <c r="H6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I6" t="n">
+        <v>2</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>benchmarks\viz_results\generated_code\viz_005.py</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>viz_006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>intermediate</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Plot time series with multiple sensor data in subplots.</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>line</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>One subplot per sensor</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>multi_ts</t>
+        </is>
+      </c>
+      <c r="G7" t="b">
+        <v>1</v>
+      </c>
+      <c r="H7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>benchmarks\viz_results\generated_code\viz_006.py</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>viz_007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>intermediate</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Create a heatmap of the multi-site temperature data.</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>heatmap</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Heatmap with sites as rows and time as columns</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>multi_site</t>
+        </is>
+      </c>
+      <c r="G8" t="b">
         <v>0</v>
       </c>
-      <c r="J6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>benchmarks\viz_results\generated_code\viz_005.py</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>reports\statistics-comparison.png</t>
-        </is>
-      </c>
-      <c r="O6" t="n">
-        <v>1</v>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>Generated 1 chart from statistics dataset showing min/mean/max comparison.</t>
+      <c r="H8" t="n">
+        <v>1</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>benchmarks\viz_results\generated_code\viz_007.py</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Visualization code execution failed: Imports are disabled in visualization code.
+Traceback (most rec</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>viz_008</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>complex</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Plot the data with missing values (NaN), handle gracefully and visualize what data is available.</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>line</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Handles NaN values appropriately</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>with_nan</t>
+        </is>
+      </c>
+      <c r="G9" t="b">
+        <v>1</v>
+      </c>
+      <c r="H9" t="n">
+        <v>1</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>benchmarks\viz_results\generated_code\viz_008.py</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>viz_009</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>complex</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Compare temperature trends across all four sites on the same plot with color differentiation.</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>line</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Multi-line chart with different colors per site</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>multi_site</t>
+        </is>
+      </c>
+      <c r="G10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H10" t="n">
+        <v>1</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>benchmarks\viz_results\generated_code\viz_009.py</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>viz_010</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>complex</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Create a combined visualization: a line chart for temperature trends with a secondary y-axis.</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>line</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Dual-axis plot with different units</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>multi_site</t>
+        </is>
+      </c>
+      <c r="G11" t="b">
+        <v>1</v>
+      </c>
+      <c r="H11" t="n">
+        <v>2</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>benchmarks\viz_results\generated_code\viz_010.py</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>viz_011</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>complex</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Visualize the distribution of measurements across channels using boxplots.</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>boxplot</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Boxplot showing distribution per channel</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>measurements</t>
+        </is>
+      </c>
+      <c r="G12" t="b">
+        <v>1</v>
+      </c>
+      <c r="H12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>benchmarks\viz_results\generated_code\viz_011.py</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>viz_012</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>complex</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Create a time series with confidence intervals or error bands.</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>line</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Time series with error bands</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>multi_ts</t>
+        </is>
+      </c>
+      <c r="G13" t="b">
+        <v>1</v>
+      </c>
+      <c r="H13" t="n">
+        <v>1</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>benchmarks\viz_results\generated_code\viz_012.py</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>viz_013</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>complex</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Generate a dashboard-style visualization with 4 subplots showing different aspects of the data.</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>multi-subplot</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>4-panel dashboard layout</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>simple_ts, wide_metrics</t>
+        </is>
+      </c>
+      <c r="G14" t="b">
+        <v>1</v>
+      </c>
+      <c r="H14" t="n">
+        <v>2</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>benchmarks\viz_results\generated_code\viz_013.py</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>viz_014</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>complex</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Visualize data where some time periods have no measurements at all.</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>line</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Handle sparse data gracefully</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>with_nan</t>
+        </is>
+      </c>
+      <c r="G15" t="b">
+        <v>1</v>
+      </c>
+      <c r="H15" t="n">
+        <v>1</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>benchmarks\viz_results\generated_code\viz_014.py</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>viz_015</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>complex</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Create a heatmap correlation matrix for numeric columns in the wide metrics data.</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>heatmap</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Correlation heatmap of numeric columns</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>wide_metrics</t>
+        </is>
+      </c>
+      <c r="G16" t="b">
+        <v>1</v>
+      </c>
+      <c r="H16" t="n">
+        <v>2</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>benchmarks\viz_results\generated_code\viz_015.py</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>viz_016</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>intermediate</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Show the time series decomposition of the simple time series data.</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>line</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Multi-panel decomposition plot</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>simple_ts</t>
+        </is>
+      </c>
+      <c r="G17" t="b">
+        <v>1</v>
+      </c>
+      <c r="H17" t="n">
+        <v>2</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>benchmarks\viz_results\generated_code\viz_016.py</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>viz_017</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>intermediate</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Create a cumulative distribution plot for the measurement readings.</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>line</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>CDF plot of readings</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>measurements</t>
+        </is>
+      </c>
+      <c r="G18" t="b">
+        <v>1</v>
+      </c>
+      <c r="H18" t="n">
+        <v>1</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>benchmarks\viz_results\generated_code\viz_017.py</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>viz_018</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>simple</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Create a histogram showing the distribution of categorical values.</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>histogram</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Histogram of category counts</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>categorical</t>
+        </is>
+      </c>
+      <c r="G19" t="b">
+        <v>1</v>
+      </c>
+      <c r="H19" t="n">
+        <v>1</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>benchmarks\viz_results\generated_code\viz_018.py</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>viz_019</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>intermediate</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Create a violin plot showing the distribution of temperature by site.</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>violin</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Violin distribution plot per site</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>multi_site</t>
+        </is>
+      </c>
+      <c r="G20" t="b">
+        <v>1</v>
+      </c>
+      <c r="H20" t="n">
+        <v>1</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>benchmarks\viz_results\generated_code\viz_019.py</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>viz_020</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>complex</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Generate an interactive-style visualization with multiple metrics aligned on time axis with proper formatting.</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>multi-line</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Complex multi-metric time series</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>multi_ts, multi_site</t>
+        </is>
+      </c>
+      <c r="G21" t="b">
+        <v>1</v>
+      </c>
+      <c r="H21" t="n">
+        <v>1</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>benchmarks\viz_results\generated_code\viz_020.py</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
     </row>

</xml_diff>